<commit_message>
docs: update candidate credentials to solo student lead Sanjai (44731076), batch 2024-2028, in presentation and runbook
</commit_message>
<xml_diff>
--- a/SIST_Student_FullStack_Project_Runbook.xlsx
+++ b/SIST_Student_FullStack_Project_Runbook.xlsx
@@ -661,7 +661,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>[REG NO - e.g. 44731034]</t>
+          <t>44731076</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>[STUDENT 2 NAME - e.g. ISHWARYA CH]</t>
+          <t>None (Solo Lead - Individual Submission)</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -683,7 +683,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>[REG NO - e.g. 44731033]</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>B.E. CSE (Artificial Intelligence) — 2nd Year</t>
+          <t>B.E. Computer Science &amp; Engineering (Artificial Intelligence)</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -705,7 +705,7 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>2023 - 2027 / Section [A1 / A2 / A3 / A4 / A5]</t>
+          <t>2024 – 2028 / 2nd Year</t>
         </is>
       </c>
     </row>
@@ -727,7 +727,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Campus Grievance Redressal &amp; SLA Auto-Escalation Web Platform</t>
+          <t>Full-Stack Web Architecture, Database Systems &amp; Process Automation</t>
         </is>
       </c>
     </row>

</xml_diff>